<commit_message>
Se actualizo el informe a febrero 2026
</commit_message>
<xml_diff>
--- a/excels/HUELGAS.xlsx
+++ b/excels/HUELGAS.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\alomeli\Documents\2024 huelgas y negociaciones 2025\Negociaciones laborales -Arturo\bases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conasamigobmx-my.sharepoint.com/personal/hector_soto_conasami_gob_mx/Documents/Escritorio/CAEL/Informes/Negociación laboral/excels/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B041BB32-475E-464F-982B-DF1048F6DE93}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{B041BB32-475E-464F-982B-DF1048F6DE93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69EA9819-42EA-4F25-AC37-7E0FDF7357F4}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{AB6C8DFA-78E8-4AC7-9423-178EB906926E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{AB6C8DFA-78E8-4AC7-9423-178EB906926E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="info" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_Hlk140572046" localSheetId="1">info!$A$1</definedName>
+    <definedName name="_Hlk188436889" localSheetId="1">info!$F$19</definedName>
+    <definedName name="_Hlk188437007" localSheetId="1">info!$B$23</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,19 +31,373 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="112">
   <si>
     <t>HUELGAS</t>
   </si>
   <si>
     <t>HUELGAS  VIGENTES</t>
+  </si>
+  <si>
+    <t>HUELGAS VIGENTES EN LA JURISDICCIÓN FEDERAL</t>
+  </si>
+  <si>
+    <t>Entidad Federativa</t>
+  </si>
+  <si>
+    <t>Empresa</t>
+  </si>
+  <si>
+    <t>Sindicato</t>
+  </si>
+  <si>
+    <t>Central Obrera</t>
+  </si>
+  <si>
+    <t>Causa</t>
+  </si>
+  <si>
+    <t>Fecha de inicio</t>
+  </si>
+  <si>
+    <t>Instancia</t>
+  </si>
+  <si>
+    <t>Personas trabajadoras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ciudad de México, Tlalpan </t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Colegio de México, A.C. Personal Administrativo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sindicato Único de Trabajadores de El Colegio de México </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otras 1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión de contrato </t>
+  </si>
+  <si>
+    <t>CFCRL-TLFAC</t>
+  </si>
+  <si>
+    <t>Más de una</t>
+  </si>
+  <si>
+    <t>entidad,</t>
+  </si>
+  <si>
+    <t>Cuauhtémoc</t>
+  </si>
+  <si>
+    <t>Nacional Monte de</t>
+  </si>
+  <si>
+    <t>Piedad, I.A.P.</t>
+  </si>
+  <si>
+    <t>Sindicato Nacional de Empleados y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trabajadores del Nacional Monte de Piedad y </t>
+  </si>
+  <si>
+    <t>de Empresas de Préstamo Prendario</t>
+  </si>
+  <si>
+    <t>CROC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Violación de </t>
+  </si>
+  <si>
+    <t>contrato</t>
+  </si>
+  <si>
+    <t>México, Tultitlán</t>
+  </si>
+  <si>
+    <t>Blurama, S.A. de</t>
+  </si>
+  <si>
+    <t>C.V.</t>
+  </si>
+  <si>
+    <t>Sindicato Nacional de Trabajadores Mineros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metalúrgicos Siderúrgicos y Similares de la </t>
+  </si>
+  <si>
+    <t>República Mexicana</t>
+  </si>
+  <si>
+    <r>
+      <t>Otras</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
+  </si>
+  <si>
+    <t>entidad</t>
+  </si>
+  <si>
+    <t>F Tapias México II,</t>
+  </si>
+  <si>
+    <t>S.A de C.V.</t>
+  </si>
+  <si>
+    <t>Embarcaciones</t>
+  </si>
+  <si>
+    <t>Monforte de Lemos</t>
+  </si>
+  <si>
+    <t>y Vigo</t>
+  </si>
+  <si>
+    <t>Orden Mexicana de Profesionales Marítimos y</t>
+  </si>
+  <si>
+    <t>Portuarios Similares y Conexo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firma de </t>
+  </si>
+  <si>
+    <t>Hidalgo,Tecozautla</t>
+  </si>
+  <si>
+    <t>RTAutomotriz, S.A. de C.V. Almacén</t>
+  </si>
+  <si>
+    <t>Sindicato Nacional de Trabajadores de landustria Metal Electrónica Mecánica y Similares de la República Mexicana</t>
+  </si>
+  <si>
+    <t>CTM</t>
+  </si>
+  <si>
+    <t>Violación de contrato</t>
+  </si>
+  <si>
+    <t>México, Toluca</t>
+  </si>
+  <si>
+    <t>Manufacturas Qualy, S.A. de C.V. Planta Toluca</t>
+  </si>
+  <si>
+    <t>Sindicato Industrial de Trabajadores Textiles</t>
+  </si>
+  <si>
+    <t>En las Ramas del Algodón Artisela Lana Y Fibras Sintéticas</t>
+  </si>
+  <si>
+    <t>Puebla, Coxcatlán</t>
+  </si>
+  <si>
+    <t>Ingenio</t>
+  </si>
+  <si>
+    <t>de</t>
+  </si>
+  <si>
+    <t>Calipam, S.A. de C.V.</t>
+  </si>
+  <si>
+    <t>Sindicato de Obreros y</t>
+  </si>
+  <si>
+    <t>Similares del</t>
+  </si>
+  <si>
+    <t>Ingenio de</t>
+  </si>
+  <si>
+    <t>Calipam</t>
+  </si>
+  <si>
+    <t>CROM</t>
+  </si>
+  <si>
+    <t>Violación de contrato ley</t>
+  </si>
+  <si>
+    <t>México,</t>
+  </si>
+  <si>
+    <t>Tianguistenco</t>
+  </si>
+  <si>
+    <t>Lerrotex, S.R.I. de c.v.</t>
+  </si>
+  <si>
+    <t>Sindicato Nacional de</t>
+  </si>
+  <si>
+    <t>Trabajadores</t>
+  </si>
+  <si>
+    <t>Adolfo López</t>
+  </si>
+  <si>
+    <t>Mateos de la Industria del Ramo Textil en General</t>
+  </si>
+  <si>
+    <t>Baja California,</t>
+  </si>
+  <si>
+    <t>Tijuana</t>
+  </si>
+  <si>
+    <t>Óxidos y</t>
+  </si>
+  <si>
+    <t>Pigmentos Mexicanos. S.A. de C.V.</t>
+  </si>
+  <si>
+    <t>Sindicato de Empleados</t>
+  </si>
+  <si>
+    <t>y Trabajadores</t>
+  </si>
+  <si>
+    <t>de la Industria el Campo y el Comercio del "Estado 29"</t>
+  </si>
+  <si>
+    <t>Baja California, Ensenada</t>
+  </si>
+  <si>
+    <t>Transportadora Maritima de Baja California,S.A de C.V.</t>
+  </si>
+  <si>
+    <t>Orden Mexicana de Profesionales Marítimos y Portuarios Similares y Conexo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Violación de contrato </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisión de  contrato </t>
+  </si>
+  <si>
+    <t>11*</t>
+  </si>
+  <si>
+    <t>Michoacán, Morelia</t>
+  </si>
+  <si>
+    <t>Alkemin, S. de R.L. C.V. División Morelia</t>
+  </si>
+  <si>
+    <t>Sindicato Nacional de Trabajadores en la Industria de Pinturas Productos Químicos Farmacéuticos</t>
+  </si>
+  <si>
+    <t>Y Alimenticios en General</t>
+  </si>
+  <si>
+    <t>y Similares en la República</t>
+  </si>
+  <si>
+    <t>Mexicana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coahuila </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mineral del Norte, S.A. de C.V. Unidad Hércules </t>
+  </si>
+  <si>
+    <t>Sindicato Nacional de Trabajadores Mineros Metalúrgicos, Siderúrgicos y Similares de la República Mexicana</t>
+  </si>
+  <si>
+    <t>Revisión salarial</t>
+  </si>
+  <si>
+    <t>Más de una entidad</t>
+  </si>
+  <si>
+    <t>Bernhard Schulte Shipmanagement México LTD, S. de R.L. de C.V.**</t>
+  </si>
+  <si>
+    <t>Tamaulipas</t>
+  </si>
+  <si>
+    <t>Palazuelos y Cia, S.C.</t>
+  </si>
+  <si>
+    <t>Sindicato Nacional de Trabajadores de Servicios y Transporte en General, Similares y Conexos de la República Mexicana</t>
+  </si>
+  <si>
+    <t>Firma de Contrato</t>
+  </si>
+  <si>
+    <t>Transportes Unidos Castañeda, S.A.P.I. de C.V.</t>
+  </si>
+  <si>
+    <t>Sindicato de Trabajadores de Todas las Ramas de la Industria y del Autotransporte C.T.M.</t>
+  </si>
+  <si>
+    <t>Tecnología Modificada, S.A. de C.V.</t>
+  </si>
+  <si>
+    <t>Sindicato Nacional Independiente de Trabajadores e Industrias y de Servicios Movimiento 20/32</t>
+  </si>
+  <si>
+    <t>Firma de contrato</t>
+  </si>
+  <si>
+    <t>Transportes Aeromar, S.A. de C.V.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sindicato Nacional de Trabajadores de la Industria del Transporte Construcción Comunicaciones Almacenaje Estibadores Mantenimiento Similares y Conexos de la República Mexicana </t>
+  </si>
+  <si>
+    <t>Asociación Sindical de Pilotos Aviadores de México y Asociación de Sobrecargos de Aviación de México</t>
+  </si>
+  <si>
+    <t>Revisión de contrato</t>
+  </si>
+  <si>
+    <t>JFCA</t>
+  </si>
+  <si>
+    <t>Guerrero</t>
+  </si>
+  <si>
+    <t>Industrial Minera México, S.A. de C.V. Unidad Taxco</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Otras </t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Noto Sans"/>
+        <family val="2"/>
+      </rPr>
+      <t>1</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -45,16 +405,48 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Noto Sans"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Noto Sans"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Noto Sans"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <vertAlign val="superscript"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Noto Sans"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF621333"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -236,26 +628,216 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -274,9 +856,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -314,7 +896,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -420,7 +1002,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -562,7 +1144,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -570,29 +1152,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E799F82-153B-4865-8E72-20431F00311A}">
-  <dimension ref="A1:C20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12"/>
-      <c r="B1" s="13" t="s">
+      <c r="A1" s="10"/>
+      <c r="B1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="9">
+      <c r="A2" s="7">
         <v>2007</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="8">
         <v>28</v>
       </c>
-      <c r="C2" s="11">
+      <c r="C2" s="9">
         <v>1</v>
       </c>
     </row>
@@ -773,28 +1355,974 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="4">
+      <c r="A19" s="2">
         <v>2024</v>
       </c>
       <c r="B19" s="1">
         <v>22</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="3">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="6">
+      <c r="A20" s="4">
         <v>2025</v>
       </c>
-      <c r="B20" s="7">
+      <c r="B20" s="5">
         <v>14</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="6">
         <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="13">
+        <v>2026</v>
+      </c>
+      <c r="B21" s="14">
+        <v>1</v>
+      </c>
+      <c r="C21" s="15">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21917D44-323C-4555-B9E3-BFB2564FBA54}">
+  <dimension ref="A1:H44"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="6" max="6" width="47.28515625" customWidth="1"/>
+    <col min="8" max="8" width="30.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="20.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="31" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+    </row>
+    <row r="2" spans="1:8" ht="69.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="37">
+        <v>46055</v>
+      </c>
+      <c r="G3" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="35">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="34"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="34"/>
+      <c r="H4" s="36"/>
+    </row>
+    <row r="5" spans="1:8" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="37">
+        <v>45930</v>
+      </c>
+      <c r="G5" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="41">
+        <v>2155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="103.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="39"/>
+      <c r="E6" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="40"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="42"/>
+    </row>
+    <row r="7" spans="1:8" ht="121.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="36"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="43"/>
+    </row>
+    <row r="8" spans="1:8" ht="103.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="37">
+        <v>45839</v>
+      </c>
+      <c r="G8" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="35">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="103.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="32"/>
+      <c r="B9" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="39"/>
+      <c r="E9" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="40"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="39"/>
+    </row>
+    <row r="10" spans="1:8" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="34"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="36"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="36"/>
+    </row>
+    <row r="11" spans="1:8" ht="120.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="37">
+        <v>45820</v>
+      </c>
+      <c r="G11" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H11" s="35">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="69" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="39"/>
+      <c r="E12" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="40"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="39"/>
+    </row>
+    <row r="13" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="23"/>
+      <c r="B13" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="25"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="40"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="39"/>
+    </row>
+    <row r="14" spans="1:8" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="23"/>
+      <c r="B14" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="25"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="39"/>
+    </row>
+    <row r="15" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="24"/>
+      <c r="B15" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="22"/>
+      <c r="D15" s="36"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="36"/>
+    </row>
+    <row r="16" spans="1:8" ht="276.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="F16" s="27">
+        <v>45777</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16" s="26">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="103.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="33" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="37">
+        <v>45723</v>
+      </c>
+      <c r="G17" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H17" s="35">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="138.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="34"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="29" t="s">
+        <v>52</v>
+      </c>
+      <c r="D18" s="36"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="36"/>
+    </row>
+    <row r="19" spans="1:8" ht="69" x14ac:dyDescent="0.25">
+      <c r="A19" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="F19" s="37">
+        <v>45642</v>
+      </c>
+      <c r="G19" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="35">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="32"/>
+      <c r="B20" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="39"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="39"/>
+    </row>
+    <row r="21" spans="1:8" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="32"/>
+      <c r="B21" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="39"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="39"/>
+    </row>
+    <row r="22" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="34"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="36"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="36"/>
+    </row>
+    <row r="23" spans="1:8" ht="51.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="B23" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="F23" s="37">
+        <v>45636</v>
+      </c>
+      <c r="G23" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H23" s="35">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="32"/>
+      <c r="C24" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D24" s="39"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="39"/>
+    </row>
+    <row r="25" spans="1:8" ht="34.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="18"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" s="39"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="39"/>
+    </row>
+    <row r="26" spans="1:8" ht="104.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="24"/>
+      <c r="B26" s="34"/>
+      <c r="C26" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="36"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="36"/>
+    </row>
+    <row r="27" spans="1:8" ht="69" x14ac:dyDescent="0.25">
+      <c r="A27" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D27" s="35" t="s">
+        <v>61</v>
+      </c>
+      <c r="E27" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" s="37">
+        <v>45569</v>
+      </c>
+      <c r="G27" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H27" s="35">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="A28" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="D28" s="39"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="39"/>
+    </row>
+    <row r="29" spans="1:8" ht="138.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="24"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D29" s="36"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="36"/>
+    </row>
+    <row r="30" spans="1:8" ht="190.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D30" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E30" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="F30" s="27">
+        <v>45513</v>
+      </c>
+      <c r="G30" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H30" s="26">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="190.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D31" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="F31" s="27">
+        <v>45513</v>
+      </c>
+      <c r="G31" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H31" s="26" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="224.25" x14ac:dyDescent="0.25">
+      <c r="A32" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="B32" s="33" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="D32" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="E32" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="F32" s="37">
+        <v>45488</v>
+      </c>
+      <c r="G32" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H32" s="35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="69" x14ac:dyDescent="0.25">
+      <c r="A33" s="32"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="D33" s="39"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="40"/>
+      <c r="G33" s="32"/>
+      <c r="H33" s="39"/>
+    </row>
+    <row r="34" spans="1:8" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="A34" s="32"/>
+      <c r="B34" s="32"/>
+      <c r="C34" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="D34" s="39"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="40"/>
+      <c r="G34" s="32"/>
+      <c r="H34" s="39"/>
+    </row>
+    <row r="35" spans="1:8" ht="18" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="34"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35" s="36"/>
+      <c r="E35" s="34"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="36"/>
+    </row>
+    <row r="36" spans="1:8" ht="259.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C36" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D36" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E36" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F36" s="27">
+        <v>45470</v>
+      </c>
+      <c r="G36" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H36" s="30">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="190.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E37" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="F37" s="27">
+        <v>45351</v>
+      </c>
+      <c r="G37" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H37" s="26">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="190.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B38" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E38" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="F38" s="27">
+        <v>45351</v>
+      </c>
+      <c r="G38" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H38" s="26">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="294" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="D39" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E39" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="F39" s="27">
+        <v>45268</v>
+      </c>
+      <c r="G39" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H39" s="26">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="207.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B40" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="D40" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="E40" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="F40" s="27">
+        <v>45262</v>
+      </c>
+      <c r="G40" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H40" s="26">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="190.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="B41" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="C41" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="D41" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E41" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="F41" s="27">
+        <v>45191</v>
+      </c>
+      <c r="G41" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H41" s="26">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C42" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="D42" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E42" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="F42" s="27">
+        <v>45001</v>
+      </c>
+      <c r="G42" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="H42" s="26">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="242.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="B43" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C43" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="D43" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="E43" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="F43" s="27">
+        <v>44973</v>
+      </c>
+      <c r="G43" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H43" s="26">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="259.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C44" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D44" s="26" t="s">
+        <v>111</v>
+      </c>
+      <c r="E44" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="F44" s="27">
+        <v>39293</v>
+      </c>
+      <c r="G44" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H44" s="26">
+        <v>403</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="53">
+    <mergeCell ref="G32:G35"/>
+    <mergeCell ref="H32:H35"/>
+    <mergeCell ref="D27:D29"/>
+    <mergeCell ref="E27:E29"/>
+    <mergeCell ref="F27:F29"/>
+    <mergeCell ref="G27:G29"/>
+    <mergeCell ref="H27:H29"/>
+    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="B32:B35"/>
+    <mergeCell ref="D32:D35"/>
+    <mergeCell ref="E32:E35"/>
+    <mergeCell ref="F32:F35"/>
+    <mergeCell ref="B23:B26"/>
+    <mergeCell ref="D23:D26"/>
+    <mergeCell ref="E23:E26"/>
+    <mergeCell ref="F23:F26"/>
+    <mergeCell ref="G23:G26"/>
+    <mergeCell ref="H23:H26"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="D19:D22"/>
+    <mergeCell ref="E19:E22"/>
+    <mergeCell ref="F19:F22"/>
+    <mergeCell ref="G19:G22"/>
+    <mergeCell ref="H19:H22"/>
+    <mergeCell ref="D11:D15"/>
+    <mergeCell ref="F11:F15"/>
+    <mergeCell ref="G11:G15"/>
+    <mergeCell ref="H11:H15"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="F5:F7"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="H5:H7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
data: actualizar insumos STPS/SCIAN a abril 2026
Refresco mensual de los archivos maestros de negociaciones, huelgas y
emplazamientos, más el nuevo tabulado SCIAN de abril 2026.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excels/HUELGAS.xlsx
+++ b/excels/HUELGAS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\alomeli\Documents\HUELGAS Y NEGOCIACIONES 2026\Negociaciones laborales -Arturo\bases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conasamigobmx-my.sharepoint.com/personal/hector_soto_conasami_gob_mx/Documents/Escritorio/CAEL/Informes/Negociación laboral/excels/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94164368-AB27-4D59-ACF0-5657E8ACD055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{2C80BD38-EF3C-4646-ACC7-465CD525431B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1DCC5FA-690E-402E-8FA1-DDE3D629BBF9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AB6C8DFA-78E8-4AC7-9423-178EB906926E}"/>
+    <workbookView xWindow="-28898" yWindow="-98" windowWidth="28996" windowHeight="16395" xr2:uid="{AB6C8DFA-78E8-4AC7-9423-178EB906926E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -569,12 +569,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E799F82-153B-4865-8E72-20431F00311A}">
   <dimension ref="A1:C21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="10"/>
       <c r="B1" s="11" t="s">
         <v>0</v>
@@ -583,7 +583,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="7">
         <v>2007</v>
       </c>
@@ -594,7 +594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <v>2008</v>
       </c>
@@ -605,7 +605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <v>2009</v>
       </c>
@@ -616,7 +616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <v>2010</v>
       </c>
@@ -627,7 +627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>2011</v>
       </c>
@@ -638,7 +638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <v>2012</v>
       </c>
@@ -649,7 +649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>2013</v>
       </c>
@@ -660,7 +660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <v>2014</v>
       </c>
@@ -671,7 +671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <v>2015</v>
       </c>
@@ -682,7 +682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <v>2016</v>
       </c>
@@ -693,7 +693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <v>2017</v>
       </c>
@@ -704,7 +704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" s="2">
         <v>2018</v>
       </c>
@@ -715,7 +715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" s="2">
         <v>2019</v>
       </c>
@@ -726,7 +726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="2">
         <v>2020</v>
       </c>
@@ -737,7 +737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" s="2">
         <v>2021</v>
       </c>
@@ -745,10 +745,10 @@
         <v>2</v>
       </c>
       <c r="C16" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <v>2022</v>
       </c>
@@ -759,7 +759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <v>2023</v>
       </c>
@@ -767,10 +767,10 @@
         <v>13</v>
       </c>
       <c r="C18" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" s="2">
         <v>2024</v>
       </c>
@@ -781,7 +781,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A20" s="4">
         <v>2025</v>
       </c>
@@ -792,15 +792,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A21" s="4">
         <v>2026</v>
       </c>
       <c r="B21" s="5">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C21" s="6">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>